<commit_message>
Prediction for 2026-09-30 (2026-08-25)
</commit_message>
<xml_diff>
--- a/outputs/rebalancing_predictions.xlsx
+++ b/outputs/rebalancing_predictions.xlsx
@@ -27,10 +27,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -49,8 +50,19 @@
     <font>
       <name val="Arial"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="00CC0000"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -82,6 +94,11 @@
         <fgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FF0000"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -101,7 +118,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
@@ -122,6 +139,13 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -487,10 +511,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I15"/>
+  <dimension ref="A1:I18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="21" customWidth="1" min="1" max="1"/>
+    <col width="50" customWidth="1" min="1" max="1"/>
     <col width="26" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
@@ -502,117 +526,69 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
+      <c r="A1" s="13" t="inlineStr">
+        <is>
+          <t>WARNING: some data could not be refreshed this run and OLDER data was used instead. This prediction may be less reliable than usual. Details below.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="14" t="inlineStr">
+        <is>
+          <t>1 symbols affected in nse_free_float</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="15" t="inlineStr">
         <is>
           <t>Review Date</t>
         </is>
       </c>
-      <c r="B1" s="3" t="inlineStr">
+      <c r="B3" s="15" t="inlineStr">
         <is>
           <t>Quarter Type</t>
         </is>
       </c>
-      <c r="C1" s="3" t="inlineStr">
+      <c r="C3" s="15" t="inlineStr">
         <is>
           <t>Adds Predicted</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
+      <c r="D3" s="15" t="inlineStr">
         <is>
           <t>Adds Actual</t>
         </is>
       </c>
-      <c r="E1" s="3" t="inlineStr">
+      <c r="E3" s="15" t="inlineStr">
         <is>
           <t>Adds Caught</t>
         </is>
       </c>
-      <c r="F1" s="3" t="inlineStr">
+      <c r="F3" s="15" t="inlineStr">
         <is>
           <t>Add Hit Rate %</t>
         </is>
       </c>
-      <c r="G1" s="3" t="inlineStr">
+      <c r="G3" s="15" t="inlineStr">
         <is>
           <t>Removes Predicted</t>
         </is>
       </c>
-      <c r="H1" s="3" t="inlineStr">
+      <c r="H3" s="15" t="inlineStr">
         <is>
           <t>Removes Actual</t>
         </is>
       </c>
-      <c r="I1" s="3" t="inlineStr">
+      <c r="I3" s="15" t="inlineStr">
         <is>
           <t>Removes Caught</t>
         </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="4" t="n">
-        <v>44926</v>
-      </c>
-      <c r="B2" s="5" t="inlineStr">
-        <is>
-          <t>Jun/Dec (fast entry)</t>
-        </is>
-      </c>
-      <c r="C2" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D2" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="E2" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="F2" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="G2" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="H2" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I2" s="5" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="4" t="n">
-        <v>45016</v>
-      </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>Mar/Sep (general review)</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="n">
-        <v>11</v>
-      </c>
-      <c r="D3" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="E3" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="F3" s="5" t="n">
-        <v>54.5</v>
-      </c>
-      <c r="G3" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="H3" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="I3" s="5" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>45107</v>
+        <v>44926</v>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
@@ -620,7 +596,7 @@
         </is>
       </c>
       <c r="C4" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D4" s="5" t="n">
         <v>0</v>
@@ -628,7 +604,9 @@
       <c r="E4" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="F4" s="5" t="inlineStr"/>
+      <c r="F4" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="G4" s="5" t="n">
         <v>0</v>
       </c>
@@ -641,7 +619,7 @@
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>45199</v>
+        <v>45016</v>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
@@ -649,22 +627,22 @@
         </is>
       </c>
       <c r="C5" s="5" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="D5" s="5" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>28.6</v>
+        <v>54.5</v>
       </c>
       <c r="G5" s="5" t="n">
         <v>0</v>
       </c>
       <c r="H5" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I5" s="5" t="n">
         <v>0</v>
@@ -672,7 +650,7 @@
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>45291</v>
+        <v>45107</v>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
@@ -680,17 +658,15 @@
         </is>
       </c>
       <c r="C6" s="5" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D6" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F6" s="5" t="n">
-        <v>50</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F6" s="5" t="inlineStr"/>
       <c r="G6" s="5" t="n">
         <v>0</v>
       </c>
@@ -703,7 +679,7 @@
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>45382</v>
+        <v>45199</v>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
@@ -711,16 +687,16 @@
         </is>
       </c>
       <c r="C7" s="5" t="n">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="D7" s="5" t="n">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="E7" s="5" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>60</v>
+        <v>28.6</v>
       </c>
       <c r="G7" s="5" t="n">
         <v>0</v>
@@ -734,7 +710,7 @@
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>45473</v>
+        <v>45291</v>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
@@ -742,16 +718,16 @@
         </is>
       </c>
       <c r="C8" s="5" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D8" s="5" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F8" s="5" t="n">
-        <v>75</v>
+        <v>50</v>
       </c>
       <c r="G8" s="5" t="n">
         <v>0</v>
@@ -765,7 +741,7 @@
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>45565</v>
+        <v>45382</v>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
@@ -773,16 +749,16 @@
         </is>
       </c>
       <c r="C9" s="5" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="D9" s="5" t="n">
         <v>13</v>
       </c>
       <c r="E9" s="5" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F9" s="5" t="n">
-        <v>73.3</v>
+        <v>60</v>
       </c>
       <c r="G9" s="5" t="n">
         <v>0</v>
@@ -796,7 +772,7 @@
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>45657</v>
+        <v>45473</v>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
@@ -804,19 +780,19 @@
         </is>
       </c>
       <c r="C10" s="5" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D10" s="5" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F10" s="5" t="n">
-        <v>14.3</v>
+        <v>75</v>
       </c>
       <c r="G10" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H10" s="5" t="n">
         <v>0</v>
@@ -827,7 +803,7 @@
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>45747</v>
+        <v>45565</v>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
@@ -835,22 +811,22 @@
         </is>
       </c>
       <c r="C11" s="5" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="D11" s="5" t="n">
         <v>13</v>
       </c>
       <c r="E11" s="5" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>65</v>
+        <v>73.3</v>
       </c>
       <c r="G11" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H11" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I11" s="5" t="n">
         <v>0</v>
@@ -858,7 +834,7 @@
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>45838</v>
+        <v>45657</v>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
@@ -866,19 +842,19 @@
         </is>
       </c>
       <c r="C12" s="5" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D12" s="5" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>83.3</v>
+        <v>14.3</v>
       </c>
       <c r="G12" s="5" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H12" s="5" t="n">
         <v>0</v>
@@ -889,7 +865,7 @@
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>45930</v>
+        <v>45747</v>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
@@ -897,22 +873,22 @@
         </is>
       </c>
       <c r="C13" s="5" t="n">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="D13" s="5" t="n">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="E13" s="5" t="n">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="F13" s="5" t="n">
-        <v>63.6</v>
+        <v>65</v>
       </c>
       <c r="G13" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H13" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I13" s="5" t="n">
         <v>0</v>
@@ -920,7 +896,7 @@
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>46022</v>
+        <v>45838</v>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
@@ -928,16 +904,16 @@
         </is>
       </c>
       <c r="C14" s="5" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D14" s="5" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F14" s="5" t="n">
-        <v>33.3</v>
+        <v>83.3</v>
       </c>
       <c r="G14" s="5" t="n">
         <v>3</v>
@@ -951,37 +927,124 @@
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
+        <v>45930</v>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Mar/Sep (general review)</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="D15" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="E15" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="F15" s="5" t="n">
+        <v>63.6</v>
+      </c>
+      <c r="G15" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="H15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="n">
+        <v>46022</v>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Jun/Dec (fast entry)</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="D16" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E16" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F16" s="5" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="G16" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="H16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="n">
         <v>46112</v>
       </c>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>Mar/Sep (general review)</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="n">
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Mar/Sep (general review)</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="n">
         <v>6</v>
       </c>
-      <c r="D15" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="E15" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F15" s="5" t="n">
+      <c r="D17" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F17" s="5" t="n">
         <v>16.7</v>
       </c>
-      <c r="G15" s="5" t="n">
+      <c r="G17" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="H15" s="5" t="n">
+      <c r="H17" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="I15" s="5" t="n">
+      <c r="I17" s="5" t="n">
         <v>2</v>
       </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="16" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Mar/Sep (general review)</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="n">
+        <v>24</v>
+      </c>
+      <c r="D18" s="5" t="n"/>
+      <c r="E18" s="5" t="n"/>
+      <c r="F18" s="5" t="n"/>
+      <c r="G18" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="H18" s="5" t="n"/>
+      <c r="I18" s="5" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:I15"/>
+  <mergeCells count="2">
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A2:I2"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1143,7 +1206,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M124"/>
+  <dimension ref="A1:M148"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
@@ -1162,67 +1225,67 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
+      <c r="A1" s="15" t="inlineStr">
         <is>
           <t>Review Date</t>
         </is>
       </c>
-      <c r="B1" s="3" t="inlineStr">
+      <c r="B1" s="15" t="inlineStr">
         <is>
           <t>Quarter Type</t>
         </is>
       </c>
-      <c r="C1" s="3" t="inlineStr">
+      <c r="C1" s="15" t="inlineStr">
         <is>
           <t>Symbol</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
+      <c r="D1" s="15" t="inlineStr">
         <is>
           <t>Company</t>
         </is>
       </c>
-      <c r="E1" s="3" t="inlineStr">
+      <c r="E1" s="15" t="inlineStr">
         <is>
           <t>Predicted</t>
         </is>
       </c>
-      <c r="F1" s="3" t="inlineStr">
+      <c r="F1" s="15" t="inlineStr">
         <is>
           <t>Actually Added</t>
         </is>
       </c>
-      <c r="G1" s="3" t="inlineStr">
+      <c r="G1" s="15" t="inlineStr">
         <is>
           <t>Outcome</t>
         </is>
       </c>
-      <c r="H1" s="3" t="inlineStr">
+      <c r="H1" s="15" t="inlineStr">
         <is>
           <t>Rank</t>
         </is>
       </c>
-      <c r="I1" s="3" t="inlineStr">
+      <c r="I1" s="15" t="inlineStr">
         <is>
           <t>Cum. Coverage %</t>
         </is>
       </c>
-      <c r="J1" s="3" t="inlineStr">
+      <c r="J1" s="15" t="inlineStr">
         <is>
           <t>Months Listed</t>
         </is>
       </c>
-      <c r="K1" s="3" t="inlineStr">
+      <c r="K1" s="15" t="inlineStr">
         <is>
           <t>Market Cap (Cr)</t>
         </is>
       </c>
-      <c r="L1" s="3" t="inlineStr">
+      <c r="L1" s="15" t="inlineStr">
         <is>
           <t>Confidence</t>
         </is>
       </c>
-      <c r="M1" s="3" t="inlineStr">
+      <c r="M1" s="15" t="inlineStr">
         <is>
           <t>Confidence Depth %</t>
         </is>
@@ -7395,6 +7458,1086 @@
       </c>
       <c r="M124" s="5" t="n">
         <v>6.3</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="16" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B125" s="5" t="inlineStr">
+        <is>
+          <t>Mar/Sep (general review)</t>
+        </is>
+      </c>
+      <c r="C125" s="5" t="inlineStr">
+        <is>
+          <t>DIVISLAB</t>
+        </is>
+      </c>
+      <c r="D125" s="5" t="inlineStr">
+        <is>
+          <t>Divi's Laboratories Ltd.</t>
+        </is>
+      </c>
+      <c r="E125" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="F125" s="5" t="n"/>
+      <c r="G125" s="5" t="n"/>
+      <c r="H125" s="5" t="n">
+        <v>40</v>
+      </c>
+      <c r="I125" s="5" t="n">
+        <v>44.5</v>
+      </c>
+      <c r="J125" s="5" t="n">
+        <v>281</v>
+      </c>
+      <c r="K125" s="5" t="n">
+        <v>228754</v>
+      </c>
+      <c r="L125" s="6" t="inlineStr">
+        <is>
+          <t>Elevated</t>
+        </is>
+      </c>
+      <c r="M125" s="5" t="n">
+        <v>49.4</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="16" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B126" s="5" t="inlineStr">
+        <is>
+          <t>Mar/Sep (general review)</t>
+        </is>
+      </c>
+      <c r="C126" s="5" t="inlineStr">
+        <is>
+          <t>ICICIAMC</t>
+        </is>
+      </c>
+      <c r="D126" s="5" t="inlineStr">
+        <is>
+          <t>ICICI Prudential Asset Management Company Ltd.</t>
+        </is>
+      </c>
+      <c r="E126" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="F126" s="5" t="n"/>
+      <c r="G126" s="5" t="n"/>
+      <c r="H126" s="5" t="n">
+        <v>58</v>
+      </c>
+      <c r="I126" s="5" t="n">
+        <v>52.4</v>
+      </c>
+      <c r="J126" s="5" t="n">
+        <v>7.4</v>
+      </c>
+      <c r="K126" s="5" t="n">
+        <v>161459</v>
+      </c>
+      <c r="L126" s="6" t="inlineStr">
+        <is>
+          <t>Elevated</t>
+        </is>
+      </c>
+      <c r="M126" s="5" t="n">
+        <v>40.4</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="16" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B127" s="5" t="inlineStr">
+        <is>
+          <t>Mar/Sep (general review)</t>
+        </is>
+      </c>
+      <c r="C127" s="5" t="inlineStr">
+        <is>
+          <t>TATACAP</t>
+        </is>
+      </c>
+      <c r="D127" s="5" t="inlineStr">
+        <is>
+          <t>Tata Capital Ltd.</t>
+        </is>
+      </c>
+      <c r="E127" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="F127" s="5" t="n"/>
+      <c r="G127" s="5" t="n"/>
+      <c r="H127" s="5" t="n">
+        <v>64</v>
+      </c>
+      <c r="I127" s="5" t="n">
+        <v>54.6</v>
+      </c>
+      <c r="J127" s="5" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="K127" s="5" t="n">
+        <v>154259</v>
+      </c>
+      <c r="L127" s="6" t="inlineStr">
+        <is>
+          <t>Elevated</t>
+        </is>
+      </c>
+      <c r="M127" s="5" t="n">
+        <v>37.9</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="16" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B128" s="5" t="inlineStr">
+        <is>
+          <t>Mar/Sep (general review)</t>
+        </is>
+      </c>
+      <c r="C128" s="5" t="inlineStr">
+        <is>
+          <t>LTM</t>
+        </is>
+      </c>
+      <c r="D128" s="5" t="inlineStr">
+        <is>
+          <t>LTM Ltd.</t>
+        </is>
+      </c>
+      <c r="E128" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="F128" s="5" t="n"/>
+      <c r="G128" s="5" t="n"/>
+      <c r="H128" s="5" t="n">
+        <v>76</v>
+      </c>
+      <c r="I128" s="5" t="n">
+        <v>58.6</v>
+      </c>
+      <c r="J128" s="5" t="n">
+        <v>120.5</v>
+      </c>
+      <c r="K128" s="5" t="n">
+        <v>134082</v>
+      </c>
+      <c r="L128" s="6" t="inlineStr">
+        <is>
+          <t>Elevated</t>
+        </is>
+      </c>
+      <c r="M128" s="5" t="n">
+        <v>33.4</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="16" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B129" s="5" t="inlineStr">
+        <is>
+          <t>Mar/Sep (general review)</t>
+        </is>
+      </c>
+      <c r="C129" s="5" t="inlineStr">
+        <is>
+          <t>GROWW</t>
+        </is>
+      </c>
+      <c r="D129" s="5" t="inlineStr">
+        <is>
+          <t>Billionbrains Garage Ventures Ltd.</t>
+        </is>
+      </c>
+      <c r="E129" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="F129" s="5" t="n"/>
+      <c r="G129" s="5" t="n"/>
+      <c r="H129" s="5" t="n">
+        <v>81</v>
+      </c>
+      <c r="I129" s="5" t="n">
+        <v>60.2</v>
+      </c>
+      <c r="J129" s="5" t="n">
+        <v>8.6</v>
+      </c>
+      <c r="K129" s="5" t="n">
+        <v>127291</v>
+      </c>
+      <c r="L129" s="6" t="inlineStr">
+        <is>
+          <t>Elevated</t>
+        </is>
+      </c>
+      <c r="M129" s="5" t="n">
+        <v>31.6</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="16" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B130" s="5" t="inlineStr">
+        <is>
+          <t>Mar/Sep (general review)</t>
+        </is>
+      </c>
+      <c r="C130" s="5" t="inlineStr">
+        <is>
+          <t>LENSKART</t>
+        </is>
+      </c>
+      <c r="D130" s="5" t="inlineStr">
+        <is>
+          <t>Lenskart Solutions Ltd.</t>
+        </is>
+      </c>
+      <c r="E130" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="F130" s="5" t="n"/>
+      <c r="G130" s="5" t="n"/>
+      <c r="H130" s="5" t="n">
+        <v>91</v>
+      </c>
+      <c r="I130" s="5" t="n">
+        <v>63</v>
+      </c>
+      <c r="J130" s="5" t="n">
+        <v>8.699999999999999</v>
+      </c>
+      <c r="K130" s="5" t="n">
+        <v>116233</v>
+      </c>
+      <c r="L130" s="6" t="inlineStr">
+        <is>
+          <t>Elevated</t>
+        </is>
+      </c>
+      <c r="M130" s="5" t="n">
+        <v>28.4</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="16" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B131" s="5" t="inlineStr">
+        <is>
+          <t>Mar/Sep (general review)</t>
+        </is>
+      </c>
+      <c r="C131" s="5" t="inlineStr">
+        <is>
+          <t>LGEINDIA</t>
+        </is>
+      </c>
+      <c r="D131" s="5" t="inlineStr">
+        <is>
+          <t>LG Electronics India Ltd.</t>
+        </is>
+      </c>
+      <c r="E131" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="F131" s="5" t="n"/>
+      <c r="G131" s="5" t="n"/>
+      <c r="H131" s="5" t="n">
+        <v>95</v>
+      </c>
+      <c r="I131" s="5" t="n">
+        <v>64.09999999999999</v>
+      </c>
+      <c r="J131" s="5" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="K131" s="5" t="n">
+        <v>114577</v>
+      </c>
+      <c r="L131" s="6" t="inlineStr">
+        <is>
+          <t>Elevated</t>
+        </is>
+      </c>
+      <c r="M131" s="5" t="n">
+        <v>27.2</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="16" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B132" s="5" t="inlineStr">
+        <is>
+          <t>Mar/Sep (general review)</t>
+        </is>
+      </c>
+      <c r="C132" s="5" t="inlineStr">
+        <is>
+          <t>MEESHO</t>
+        </is>
+      </c>
+      <c r="D132" s="5" t="inlineStr">
+        <is>
+          <t>Meesho Ltd.</t>
+        </is>
+      </c>
+      <c r="E132" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="F132" s="5" t="n"/>
+      <c r="G132" s="5" t="n"/>
+      <c r="H132" s="5" t="n">
+        <v>123</v>
+      </c>
+      <c r="I132" s="5" t="n">
+        <v>71</v>
+      </c>
+      <c r="J132" s="5" t="n">
+        <v>7.7</v>
+      </c>
+      <c r="K132" s="5" t="n">
+        <v>96383</v>
+      </c>
+      <c r="L132" s="8" t="inlineStr">
+        <is>
+          <t>Watch</t>
+        </is>
+      </c>
+      <c r="M132" s="5" t="n">
+        <v>19.3</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="16" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B133" s="5" t="inlineStr">
+        <is>
+          <t>Mar/Sep (general review)</t>
+        </is>
+      </c>
+      <c r="C133" s="5" t="inlineStr">
+        <is>
+          <t>AUROPHARMA</t>
+        </is>
+      </c>
+      <c r="D133" s="5" t="inlineStr">
+        <is>
+          <t>Aurobindo Pharma Ltd.</t>
+        </is>
+      </c>
+      <c r="E133" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="F133" s="5" t="n"/>
+      <c r="G133" s="5" t="n"/>
+      <c r="H133" s="5" t="n">
+        <v>127</v>
+      </c>
+      <c r="I133" s="5" t="n">
+        <v>71.90000000000001</v>
+      </c>
+      <c r="J133" s="5" t="n">
+        <v>312.8</v>
+      </c>
+      <c r="K133" s="5" t="n">
+        <v>92877</v>
+      </c>
+      <c r="L133" s="8" t="inlineStr">
+        <is>
+          <t>Watch</t>
+        </is>
+      </c>
+      <c r="M133" s="5" t="n">
+        <v>18.3</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="16" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B134" s="5" t="inlineStr">
+        <is>
+          <t>Mar/Sep (general review)</t>
+        </is>
+      </c>
+      <c r="C134" s="5" t="inlineStr">
+        <is>
+          <t>SHREECEM</t>
+        </is>
+      </c>
+      <c r="D134" s="5" t="inlineStr">
+        <is>
+          <t>Shree Cement Ltd.</t>
+        </is>
+      </c>
+      <c r="E134" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="F134" s="5" t="n"/>
+      <c r="G134" s="5" t="n"/>
+      <c r="H134" s="5" t="n">
+        <v>130</v>
+      </c>
+      <c r="I134" s="5" t="n">
+        <v>72.5</v>
+      </c>
+      <c r="J134" s="5" t="n">
+        <v>375.6</v>
+      </c>
+      <c r="K134" s="5" t="n">
+        <v>88109</v>
+      </c>
+      <c r="L134" s="8" t="inlineStr">
+        <is>
+          <t>Watch</t>
+        </is>
+      </c>
+      <c r="M134" s="5" t="n">
+        <v>17.6</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="16" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B135" s="5" t="inlineStr">
+        <is>
+          <t>Mar/Sep (general review)</t>
+        </is>
+      </c>
+      <c r="C135" s="5" t="inlineStr">
+        <is>
+          <t>ASTERDM</t>
+        </is>
+      </c>
+      <c r="D135" s="5" t="inlineStr">
+        <is>
+          <t>Aster DM Healthcare Ltd.</t>
+        </is>
+      </c>
+      <c r="E135" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="F135" s="5" t="n"/>
+      <c r="G135" s="5" t="n"/>
+      <c r="H135" s="5" t="n">
+        <v>169</v>
+      </c>
+      <c r="I135" s="5" t="n">
+        <v>79.5</v>
+      </c>
+      <c r="J135" s="5" t="n">
+        <v>101.2</v>
+      </c>
+      <c r="K135" s="5" t="n">
+        <v>66535</v>
+      </c>
+      <c r="L135" s="8" t="inlineStr">
+        <is>
+          <t>Watch</t>
+        </is>
+      </c>
+      <c r="M135" s="5" t="n">
+        <v>9.699999999999999</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="16" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B136" s="5" t="inlineStr">
+        <is>
+          <t>Mar/Sep (general review)</t>
+        </is>
+      </c>
+      <c r="C136" s="5" t="inlineStr">
+        <is>
+          <t>WELCORP</t>
+        </is>
+      </c>
+      <c r="D136" s="5" t="inlineStr">
+        <is>
+          <t>Welspun Corp Ltd.</t>
+        </is>
+      </c>
+      <c r="E136" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="F136" s="5" t="n"/>
+      <c r="G136" s="5" t="n"/>
+      <c r="H136" s="5" t="n">
+        <v>175</v>
+      </c>
+      <c r="I136" s="5" t="n">
+        <v>80.40000000000001</v>
+      </c>
+      <c r="J136" s="5" t="n">
+        <v>254.5</v>
+      </c>
+      <c r="K136" s="5" t="n">
+        <v>62914</v>
+      </c>
+      <c r="L136" s="8" t="inlineStr">
+        <is>
+          <t>Watch</t>
+        </is>
+      </c>
+      <c r="M136" s="5" t="n">
+        <v>8.6</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="16" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B137" s="5" t="inlineStr">
+        <is>
+          <t>Mar/Sep (general review)</t>
+        </is>
+      </c>
+      <c r="C137" s="5" t="inlineStr">
+        <is>
+          <t>RADICO</t>
+        </is>
+      </c>
+      <c r="D137" s="5" t="inlineStr">
+        <is>
+          <t>Radico Khaitan Ltd</t>
+        </is>
+      </c>
+      <c r="E137" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="F137" s="5" t="n"/>
+      <c r="G137" s="5" t="n"/>
+      <c r="H137" s="5" t="n">
+        <v>179</v>
+      </c>
+      <c r="I137" s="5" t="n">
+        <v>81</v>
+      </c>
+      <c r="J137" s="5" t="n">
+        <v>277.8</v>
+      </c>
+      <c r="K137" s="5" t="n">
+        <v>62180</v>
+      </c>
+      <c r="L137" s="8" t="inlineStr">
+        <is>
+          <t>Watch</t>
+        </is>
+      </c>
+      <c r="M137" s="5" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="16" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B138" s="5" t="inlineStr">
+        <is>
+          <t>Mar/Sep (general review)</t>
+        </is>
+      </c>
+      <c r="C138" s="5" t="inlineStr">
+        <is>
+          <t>FACT</t>
+        </is>
+      </c>
+      <c r="D138" s="5" t="inlineStr">
+        <is>
+          <t>Fertilisers and Chemicals Travancore Ltd.</t>
+        </is>
+      </c>
+      <c r="E138" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="F138" s="5" t="n"/>
+      <c r="G138" s="5" t="n"/>
+      <c r="H138" s="5" t="n">
+        <v>188</v>
+      </c>
+      <c r="I138" s="5" t="n">
+        <v>82.3</v>
+      </c>
+      <c r="J138" s="5" t="n">
+        <v>376.1</v>
+      </c>
+      <c r="K138" s="5" t="n">
+        <v>57509</v>
+      </c>
+      <c r="L138" s="8" t="inlineStr">
+        <is>
+          <t>Watch</t>
+        </is>
+      </c>
+      <c r="M138" s="5" t="n">
+        <v>6.5</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="16" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B139" s="5" t="inlineStr">
+        <is>
+          <t>Mar/Sep (general review)</t>
+        </is>
+      </c>
+      <c r="C139" s="5" t="inlineStr">
+        <is>
+          <t>ATHERENERG</t>
+        </is>
+      </c>
+      <c r="D139" s="5" t="inlineStr">
+        <is>
+          <t>Ather Energy Ltd.</t>
+        </is>
+      </c>
+      <c r="E139" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="F139" s="5" t="n"/>
+      <c r="G139" s="5" t="n"/>
+      <c r="H139" s="5" t="n">
+        <v>190</v>
+      </c>
+      <c r="I139" s="5" t="n">
+        <v>82.5</v>
+      </c>
+      <c r="J139" s="5" t="n">
+        <v>14.8</v>
+      </c>
+      <c r="K139" s="5" t="n">
+        <v>56933</v>
+      </c>
+      <c r="L139" s="8" t="inlineStr">
+        <is>
+          <t>Watch</t>
+        </is>
+      </c>
+      <c r="M139" s="5" t="n">
+        <v>6.2</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="16" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B140" s="5" t="inlineStr">
+        <is>
+          <t>Mar/Sep (general review)</t>
+        </is>
+      </c>
+      <c r="C140" s="5" t="inlineStr">
+        <is>
+          <t>ABBOTINDIA</t>
+        </is>
+      </c>
+      <c r="D140" s="5" t="inlineStr">
+        <is>
+          <t>Abbott India Ltd.</t>
+        </is>
+      </c>
+      <c r="E140" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="F140" s="5" t="n"/>
+      <c r="G140" s="5" t="n"/>
+      <c r="H140" s="5" t="n">
+        <v>193</v>
+      </c>
+      <c r="I140" s="5" t="n">
+        <v>82.90000000000001</v>
+      </c>
+      <c r="J140" s="5" t="n">
+        <v>198.9</v>
+      </c>
+      <c r="K140" s="5" t="n">
+        <v>56151</v>
+      </c>
+      <c r="L140" s="8" t="inlineStr">
+        <is>
+          <t>Watch</t>
+        </is>
+      </c>
+      <c r="M140" s="5" t="n">
+        <v>5.8</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="16" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B141" s="5" t="inlineStr">
+        <is>
+          <t>Mar/Sep (general review)</t>
+        </is>
+      </c>
+      <c r="C141" s="5" t="inlineStr">
+        <is>
+          <t>ANTHEM</t>
+        </is>
+      </c>
+      <c r="D141" s="5" t="inlineStr">
+        <is>
+          <t>Anthem Biosciences Ltd.</t>
+        </is>
+      </c>
+      <c r="E141" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="F141" s="5" t="n"/>
+      <c r="G141" s="5" t="n"/>
+      <c r="H141" s="5" t="n">
+        <v>208</v>
+      </c>
+      <c r="I141" s="5" t="n">
+        <v>84.7</v>
+      </c>
+      <c r="J141" s="5" t="n">
+        <v>12.3</v>
+      </c>
+      <c r="K141" s="5" t="n">
+        <v>49352</v>
+      </c>
+      <c r="L141" s="8" t="inlineStr">
+        <is>
+          <t>Watch</t>
+        </is>
+      </c>
+      <c r="M141" s="5" t="n">
+        <v>3.7</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="16" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B142" s="5" t="inlineStr">
+        <is>
+          <t>Mar/Sep (general review)</t>
+        </is>
+      </c>
+      <c r="C142" s="5" t="inlineStr">
+        <is>
+          <t>AEGISLOG</t>
+        </is>
+      </c>
+      <c r="D142" s="5" t="inlineStr">
+        <is>
+          <t>Aegis Logistics Ltd.</t>
+        </is>
+      </c>
+      <c r="E142" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="F142" s="5" t="n"/>
+      <c r="G142" s="5" t="n"/>
+      <c r="H142" s="5" t="n">
+        <v>216</v>
+      </c>
+      <c r="I142" s="5" t="n">
+        <v>85.59999999999999</v>
+      </c>
+      <c r="J142" s="5" t="n">
+        <v>364.3</v>
+      </c>
+      <c r="K142" s="5" t="n">
+        <v>46795</v>
+      </c>
+      <c r="L142" s="8" t="inlineStr">
+        <is>
+          <t>Watch</t>
+        </is>
+      </c>
+      <c r="M142" s="5" t="n">
+        <v>2.7</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="16" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B143" s="5" t="inlineStr">
+        <is>
+          <t>Mar/Sep (general review)</t>
+        </is>
+      </c>
+      <c r="C143" s="5" t="inlineStr">
+        <is>
+          <t>GLAND</t>
+        </is>
+      </c>
+      <c r="D143" s="5" t="inlineStr">
+        <is>
+          <t>Gland Pharma Ltd.</t>
+        </is>
+      </c>
+      <c r="E143" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="F143" s="5" t="n"/>
+      <c r="G143" s="5" t="n"/>
+      <c r="H143" s="5" t="n">
+        <v>217</v>
+      </c>
+      <c r="I143" s="5" t="n">
+        <v>85.8</v>
+      </c>
+      <c r="J143" s="5" t="n">
+        <v>68.40000000000001</v>
+      </c>
+      <c r="K143" s="5" t="n">
+        <v>46432</v>
+      </c>
+      <c r="L143" s="8" t="inlineStr">
+        <is>
+          <t>Watch</t>
+        </is>
+      </c>
+      <c r="M143" s="5" t="n">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="16" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B144" s="5" t="inlineStr">
+        <is>
+          <t>Mar/Sep (general review)</t>
+        </is>
+      </c>
+      <c r="C144" s="5" t="inlineStr">
+        <is>
+          <t>AJANTPHARM</t>
+        </is>
+      </c>
+      <c r="D144" s="5" t="inlineStr">
+        <is>
+          <t>Ajanta Pharmaceuticals Ltd.</t>
+        </is>
+      </c>
+      <c r="E144" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="F144" s="5" t="n"/>
+      <c r="G144" s="5" t="n"/>
+      <c r="H144" s="5" t="n">
+        <v>222</v>
+      </c>
+      <c r="I144" s="5" t="n">
+        <v>86.3</v>
+      </c>
+      <c r="J144" s="5" t="n">
+        <v>314.4</v>
+      </c>
+      <c r="K144" s="5" t="n">
+        <v>44312</v>
+      </c>
+      <c r="L144" s="8" t="inlineStr">
+        <is>
+          <t>Watch</t>
+        </is>
+      </c>
+      <c r="M144" s="5" t="n">
+        <v>1.9</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="16" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B145" s="5" t="inlineStr">
+        <is>
+          <t>Mar/Sep (general review)</t>
+        </is>
+      </c>
+      <c r="C145" s="5" t="inlineStr">
+        <is>
+          <t>NAVINFLUOR</t>
+        </is>
+      </c>
+      <c r="D145" s="5" t="inlineStr">
+        <is>
+          <t>Navin Fluorine International Ltd.</t>
+        </is>
+      </c>
+      <c r="E145" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="F145" s="5" t="n"/>
+      <c r="G145" s="5" t="n"/>
+      <c r="H145" s="5" t="n">
+        <v>224</v>
+      </c>
+      <c r="I145" s="5" t="n">
+        <v>86.5</v>
+      </c>
+      <c r="J145" s="5" t="n">
+        <v>230.3</v>
+      </c>
+      <c r="K145" s="5" t="n">
+        <v>42074</v>
+      </c>
+      <c r="L145" s="8" t="inlineStr">
+        <is>
+          <t>Watch</t>
+        </is>
+      </c>
+      <c r="M145" s="5" t="n">
+        <v>1.7</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="16" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B146" s="5" t="inlineStr">
+        <is>
+          <t>Mar/Sep (general review)</t>
+        </is>
+      </c>
+      <c r="C146" s="5" t="inlineStr">
+        <is>
+          <t>JKCEMENT</t>
+        </is>
+      </c>
+      <c r="D146" s="5" t="inlineStr">
+        <is>
+          <t>J.K. Cement Ltd.</t>
+        </is>
+      </c>
+      <c r="E146" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="F146" s="5" t="n"/>
+      <c r="G146" s="5" t="n"/>
+      <c r="H146" s="5" t="n">
+        <v>229</v>
+      </c>
+      <c r="I146" s="5" t="n">
+        <v>87</v>
+      </c>
+      <c r="J146" s="5" t="n">
+        <v>244.9</v>
+      </c>
+      <c r="K146" s="5" t="n">
+        <v>40122</v>
+      </c>
+      <c r="L146" s="8" t="inlineStr">
+        <is>
+          <t>Watch</t>
+        </is>
+      </c>
+      <c r="M146" s="5" t="n">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="16" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B147" s="5" t="inlineStr">
+        <is>
+          <t>Mar/Sep (general review)</t>
+        </is>
+      </c>
+      <c r="C147" s="5" t="inlineStr">
+        <is>
+          <t>CPPLUS</t>
+        </is>
+      </c>
+      <c r="D147" s="5" t="inlineStr">
+        <is>
+          <t>Aditya Infotech Ltd.</t>
+        </is>
+      </c>
+      <c r="E147" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="F147" s="5" t="n"/>
+      <c r="G147" s="5" t="n"/>
+      <c r="H147" s="5" t="n">
+        <v>230</v>
+      </c>
+      <c r="I147" s="5" t="n">
+        <v>87.09999999999999</v>
+      </c>
+      <c r="J147" s="5" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="K147" s="5" t="n">
+        <v>40094</v>
+      </c>
+      <c r="L147" s="8" t="inlineStr">
+        <is>
+          <t>Watch</t>
+        </is>
+      </c>
+      <c r="M147" s="5" t="n">
+        <v>1.1</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="16" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B148" s="5" t="inlineStr">
+        <is>
+          <t>Mar/Sep (general review)</t>
+        </is>
+      </c>
+      <c r="C148" s="5" t="inlineStr">
+        <is>
+          <t>KPRMILL</t>
+        </is>
+      </c>
+      <c r="D148" s="5" t="inlineStr">
+        <is>
+          <t>K.P.R. Mill Ltd.</t>
+        </is>
+      </c>
+      <c r="E148" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="F148" s="5" t="n"/>
+      <c r="G148" s="5" t="n"/>
+      <c r="H148" s="5" t="n">
+        <v>238</v>
+      </c>
+      <c r="I148" s="5" t="n">
+        <v>87.8</v>
+      </c>
+      <c r="J148" s="5" t="n">
+        <v>227.4</v>
+      </c>
+      <c r="K148" s="5" t="n">
+        <v>38174</v>
+      </c>
+      <c r="L148" s="8" t="inlineStr">
+        <is>
+          <t>Watch</t>
+        </is>
+      </c>
+      <c r="M148" s="5" t="n">
+        <v>0.2</v>
       </c>
     </row>
   </sheetData>
@@ -7409,7 +8552,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L18"/>
+  <dimension ref="A1:L21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
@@ -7427,62 +8570,62 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
+      <c r="A1" s="15" t="inlineStr">
         <is>
           <t>Review Date</t>
         </is>
       </c>
-      <c r="B1" s="3" t="inlineStr">
+      <c r="B1" s="15" t="inlineStr">
         <is>
           <t>Quarter Type</t>
         </is>
       </c>
-      <c r="C1" s="3" t="inlineStr">
+      <c r="C1" s="15" t="inlineStr">
         <is>
           <t>Symbol</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
+      <c r="D1" s="15" t="inlineStr">
         <is>
           <t>Company</t>
         </is>
       </c>
-      <c r="E1" s="3" t="inlineStr">
+      <c r="E1" s="15" t="inlineStr">
         <is>
           <t>Predicted</t>
         </is>
       </c>
-      <c r="F1" s="3" t="inlineStr">
+      <c r="F1" s="15" t="inlineStr">
         <is>
           <t>Actually Removed</t>
         </is>
       </c>
-      <c r="G1" s="3" t="inlineStr">
+      <c r="G1" s="15" t="inlineStr">
         <is>
           <t>Outcome</t>
         </is>
       </c>
-      <c r="H1" s="3" t="inlineStr">
+      <c r="H1" s="15" t="inlineStr">
         <is>
           <t>Rank</t>
         </is>
       </c>
-      <c r="I1" s="3" t="inlineStr">
+      <c r="I1" s="15" t="inlineStr">
         <is>
           <t>Cum. Coverage %</t>
         </is>
       </c>
-      <c r="J1" s="3" t="inlineStr">
+      <c r="J1" s="15" t="inlineStr">
         <is>
           <t>Market Cap (Cr)</t>
         </is>
       </c>
-      <c r="K1" s="3" t="inlineStr">
+      <c r="K1" s="15" t="inlineStr">
         <is>
           <t>Confidence</t>
         </is>
       </c>
-      <c r="L1" s="3" t="inlineStr">
+      <c r="L1" s="15" t="inlineStr">
         <is>
           <t>Confidence Depth %</t>
         </is>
@@ -8288,6 +9431,132 @@
       </c>
       <c r="L18" s="5" t="n">
         <v>3.6</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="16" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Mar/Sep (general review)</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>BATAINDIA</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>Bata India Ltd.</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="F19" s="5" t="n"/>
+      <c r="G19" s="5" t="n"/>
+      <c r="H19" s="5" t="n">
+        <v>487</v>
+      </c>
+      <c r="I19" s="5" t="n">
+        <v>99.8</v>
+      </c>
+      <c r="J19" s="5" t="n">
+        <v>8782</v>
+      </c>
+      <c r="K19" s="7" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L19" s="5" t="n">
+        <v>90.3</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="16" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Mar/Sep (general review)</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>WHIRLPOOL</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>Whirlpool of India Ltd.</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="F20" s="5" t="n"/>
+      <c r="G20" s="5" t="n"/>
+      <c r="H20" s="5" t="n">
+        <v>477</v>
+      </c>
+      <c r="I20" s="5" t="n">
+        <v>99.59999999999999</v>
+      </c>
+      <c r="J20" s="5" t="n">
+        <v>9704</v>
+      </c>
+      <c r="K20" s="7" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L20" s="5" t="n">
+        <v>79.40000000000001</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="16" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>Mar/Sep (general review)</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>INDIACEM</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>India Cements Ltd.</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="F21" s="5" t="n"/>
+      <c r="G21" s="5" t="n"/>
+      <c r="H21" s="5" t="n">
+        <v>453</v>
+      </c>
+      <c r="I21" s="5" t="n">
+        <v>99</v>
+      </c>
+      <c r="J21" s="5" t="n">
+        <v>11294</v>
+      </c>
+      <c r="K21" s="6" t="inlineStr">
+        <is>
+          <t>Elevated</t>
+        </is>
+      </c>
+      <c r="L21" s="5" t="n">
+        <v>49.8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>